<commit_message>
Quartz sync: Aug 27, 2025, 7:58 PM
</commit_message>
<xml_diff>
--- a/content/Economia politica/3°/File/EconomiaPolitica.xlsx
+++ b/content/Economia politica/3°/File/EconomiaPolitica.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utente\Desktop\AppuntiScuola\content\Economia politica\3°\File\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5E3DA07-5046-4D90-AEFF-6CC7519C851D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A1C94B-4A4E-4279-A006-BF2FA73F9D8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6A4CFDC2-E119-4457-B5F6-44896FCEDC5E}"/>
   </bookViews>
   <sheets>
     <sheet name="Costi" sheetId="3" r:id="rId1"/>
-    <sheet name="Utilità" sheetId="2" r:id="rId2"/>
-    <sheet name="Saggio marginale di sostiuzione" sheetId="1" r:id="rId3"/>
+    <sheet name="Ricavi" sheetId="4" r:id="rId2"/>
+    <sheet name="Utilità" sheetId="2" r:id="rId3"/>
+    <sheet name="Saggio marginale di sostiuzione" sheetId="1" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="34">
   <si>
     <t>A</t>
   </si>
@@ -133,6 +134,12 @@
   <si>
     <t>I costi crescono entrambi, seppure di intensità differenti; Il motivo è che i costi medi hanno i costi fissi che attenuano la crescita</t>
   </si>
+  <si>
+    <t>Ricavi totali</t>
+  </si>
+  <si>
+    <t>Ricavi marginali</t>
+  </si>
 </sst>
 </file>
 
@@ -970,7 +977,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -1119,6 +1126,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3255,6 +3265,228 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B351482E-B0ED-4D3C-A8D2-34B53834CE6E}">
+  <dimension ref="B1:F12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.42578125" customWidth="1"/>
+    <col min="6" max="6" width="24.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="45" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="46" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="41">
+        <v>0</v>
+      </c>
+      <c r="C3" s="42">
+        <f>B3*Costi!$C$16</f>
+        <v>0</v>
+      </c>
+      <c r="D3" s="43" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="43" t="str">
+        <f>Costi!G3</f>
+        <v>-</v>
+      </c>
+      <c r="F3" s="44" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="24">
+        <v>1</v>
+      </c>
+      <c r="C4" s="42">
+        <f>B4*Costi!$C$16</f>
+        <v>45</v>
+      </c>
+      <c r="D4" s="4">
+        <f>C4-C3</f>
+        <v>45</v>
+      </c>
+      <c r="E4" s="43">
+        <f>Costi!G4</f>
+        <v>20</v>
+      </c>
+      <c r="F4" s="40" t="str">
+        <f>IF(D4=E4,"Ottimo economico","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="24">
+        <v>2</v>
+      </c>
+      <c r="C5" s="42">
+        <f>B5*Costi!$C$16</f>
+        <v>90</v>
+      </c>
+      <c r="D5" s="4">
+        <f t="shared" ref="D5:D11" si="0">C5-C4</f>
+        <v>45</v>
+      </c>
+      <c r="E5" s="43">
+        <f>Costi!G5</f>
+        <v>10</v>
+      </c>
+      <c r="F5" s="40" t="str">
+        <f t="shared" ref="F5:F11" si="1">IF(D5=E5,"Ottimo economico","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="24">
+        <v>3</v>
+      </c>
+      <c r="C6" s="42">
+        <f>B6*Costi!$C$16</f>
+        <v>135</v>
+      </c>
+      <c r="D6" s="4">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="E6" s="43">
+        <f>Costi!G6</f>
+        <v>7.5</v>
+      </c>
+      <c r="F6" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="24">
+        <v>4</v>
+      </c>
+      <c r="C7" s="42">
+        <f>B7*Costi!$C$16</f>
+        <v>180</v>
+      </c>
+      <c r="D7" s="4">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="E7" s="43">
+        <f>Costi!G7</f>
+        <v>5</v>
+      </c>
+      <c r="F7" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="24">
+        <v>5</v>
+      </c>
+      <c r="C8" s="42">
+        <f>B8*Costi!$C$16</f>
+        <v>225</v>
+      </c>
+      <c r="D8" s="4">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="E8" s="43">
+        <f>Costi!G8</f>
+        <v>7.5</v>
+      </c>
+      <c r="F8" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="24">
+        <v>6</v>
+      </c>
+      <c r="C9" s="42">
+        <f>B9*Costi!$C$16</f>
+        <v>270</v>
+      </c>
+      <c r="D9" s="4">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="E9" s="43">
+        <f>Costi!G9</f>
+        <v>30</v>
+      </c>
+      <c r="F9" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="24">
+        <v>7</v>
+      </c>
+      <c r="C10" s="42">
+        <f>B10*Costi!$C$16</f>
+        <v>315</v>
+      </c>
+      <c r="D10" s="4">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="E10" s="43">
+        <f>Costi!G10</f>
+        <v>45</v>
+      </c>
+      <c r="F10" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>Ottimo economico</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="25">
+        <v>8</v>
+      </c>
+      <c r="C11" s="17">
+        <f>B11*Costi!$C$16</f>
+        <v>360</v>
+      </c>
+      <c r="D11" s="17">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="E11" s="69">
+        <f>Costi!G11</f>
+        <v>75</v>
+      </c>
+      <c r="F11" s="51" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55F4C1D9-4468-40EE-AEC1-05AC83165741}">
   <dimension ref="B1:H13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3511,7 +3743,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A626EAAB-1106-4797-A563-A5DAD61BAF0D}">
   <dimension ref="C2:K22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Quartz sync: Aug 28, 2025, 3:39 PM
</commit_message>
<xml_diff>
--- a/content/Economia politica/3°/File/EconomiaPolitica.xlsx
+++ b/content/Economia politica/3°/File/EconomiaPolitica.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utente\Desktop\AppuntiScuola\content\Economia politica\3°\File\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A1C94B-4A4E-4279-A006-BF2FA73F9D8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7836B659-D0FA-4DD3-9A78-DBDE00BDB699}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6A4CFDC2-E119-4457-B5F6-44896FCEDC5E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6A4CFDC2-E119-4457-B5F6-44896FCEDC5E}"/>
   </bookViews>
   <sheets>
     <sheet name="Costi" sheetId="3" r:id="rId1"/>
-    <sheet name="Ricavi" sheetId="4" r:id="rId2"/>
-    <sheet name="Utilità" sheetId="2" r:id="rId3"/>
-    <sheet name="Saggio marginale di sostiuzione" sheetId="1" r:id="rId4"/>
+    <sheet name="Impresa monopolistica" sheetId="5" r:id="rId2"/>
+    <sheet name="Ricavi" sheetId="4" r:id="rId3"/>
+    <sheet name="Utilità" sheetId="2" r:id="rId4"/>
+    <sheet name="Saggio marginale di sostiuzione" sheetId="1" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="35">
   <si>
     <t>A</t>
   </si>
@@ -140,6 +141,9 @@
   <si>
     <t>Ricavi marginali</t>
   </si>
+  <si>
+    <t>ExtraProfitto</t>
+  </si>
 </sst>
 </file>
 
@@ -211,7 +215,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="55">
+  <borders count="57">
     <border>
       <left/>
       <right/>
@@ -929,47 +933,65 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color auto="1"/>
+      <left style="thick">
+        <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color auto="1"/>
+      <right style="thin">
+        <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color auto="1"/>
+      <right style="thin">
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color auto="1"/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -977,7 +999,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -1067,27 +1089,27 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="53" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1127,9 +1149,11 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -3164,11 +3188,11 @@
         <f t="shared" si="2"/>
         <v>75</v>
       </c>
-      <c r="H11" s="50" t="str">
+      <c r="H11" s="47" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="I11" s="51" t="str">
+      <c r="I11" s="48" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -3177,49 +3201,59 @@
       <c r="H12" s="38"/>
       <c r="I12" s="38"/>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B13" s="47" t="s">
+    <row r="13" spans="2:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="50" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="53">
+      <c r="C13" s="51">
         <v>100</v>
       </c>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="48" t="s">
+      <c r="B14" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="54">
+      <c r="C14" s="53">
         <f>INDEX(F4:F11, MATCH("Punto di fuga", H4:H11, 0))</f>
         <v>30</v>
       </c>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B15" s="48" t="s">
+      <c r="B15" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="54">
+      <c r="C15" s="53">
         <f>INDEX(B3:B11, MATCH(C14, G3:G11, 0))</f>
         <v>6</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="48" t="s">
+      <c r="B16" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="55">
+      <c r="C16" s="54">
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="49" t="s">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" s="52" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="52">
+      <c r="C17" s="53">
         <f>IF(C16&lt;C14,"Si esce dal mercato",INDEX(B3:B11,MATCH("Ottimo economico",I3:I11,0)))</f>
         <v>7</v>
       </c>
     </row>
+    <row r="18" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="55" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="31">
+        <f>VLOOKUP(Costi!C17,Ricavi!B2:F11,2,FALSE)-VLOOKUP(Costi!C17,Costi!B2:I11,4,FALSE)</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>25</v>
@@ -3265,6 +3299,313 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{190A7578-06CC-40A7-B0C7-10162DA7FB2E}">
+  <dimension ref="B1:G16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="45" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="36" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="36" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="41">
+        <v>0</v>
+      </c>
+      <c r="C3" s="42">
+        <f>$C$16</f>
+        <v>100</v>
+      </c>
+      <c r="D3" s="42">
+        <v>0</v>
+      </c>
+      <c r="E3" s="42">
+        <f t="shared" ref="E3:E11" si="0">C3+D3</f>
+        <v>100</v>
+      </c>
+      <c r="F3" s="43" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="43" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B4" s="24">
+        <v>1</v>
+      </c>
+      <c r="C4" s="42">
+        <f t="shared" ref="C4:C13" si="1">$C$16</f>
+        <v>100</v>
+      </c>
+      <c r="D4" s="4">
+        <v>20</v>
+      </c>
+      <c r="E4" s="4">
+        <f t="shared" si="0"/>
+        <v>120</v>
+      </c>
+      <c r="F4" s="4">
+        <f>ROUNDDOWN(E4/B4,1)</f>
+        <v>120</v>
+      </c>
+      <c r="G4" s="4">
+        <f t="shared" ref="G4:G11" si="2">E4-E3</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" s="24">
+        <v>2</v>
+      </c>
+      <c r="C5" s="42">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="D5" s="4">
+        <v>30</v>
+      </c>
+      <c r="E5" s="4">
+        <f t="shared" si="0"/>
+        <v>130</v>
+      </c>
+      <c r="F5" s="4">
+        <f t="shared" ref="F5:F11" si="3">ROUNDDOWN(E5/B5,1)</f>
+        <v>65</v>
+      </c>
+      <c r="G5" s="4">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6" s="24">
+        <v>3</v>
+      </c>
+      <c r="C6" s="42">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="D6" s="4">
+        <v>37.5</v>
+      </c>
+      <c r="E6" s="4">
+        <f t="shared" si="0"/>
+        <v>137.5</v>
+      </c>
+      <c r="F6" s="4">
+        <f t="shared" si="3"/>
+        <v>45.8</v>
+      </c>
+      <c r="G6" s="4">
+        <f t="shared" si="2"/>
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="24">
+        <v>4</v>
+      </c>
+      <c r="C7" s="42">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="D7" s="4">
+        <v>42.5</v>
+      </c>
+      <c r="E7" s="4">
+        <f t="shared" si="0"/>
+        <v>142.5</v>
+      </c>
+      <c r="F7" s="4">
+        <f t="shared" si="3"/>
+        <v>35.6</v>
+      </c>
+      <c r="G7" s="4">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="24">
+        <v>5</v>
+      </c>
+      <c r="C8" s="42">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="D8" s="4">
+        <v>50</v>
+      </c>
+      <c r="E8" s="4">
+        <f t="shared" si="0"/>
+        <v>150</v>
+      </c>
+      <c r="F8" s="4">
+        <f t="shared" si="3"/>
+        <v>30</v>
+      </c>
+      <c r="G8" s="4">
+        <f t="shared" si="2"/>
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="24">
+        <v>6</v>
+      </c>
+      <c r="C9" s="42">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="D9" s="4">
+        <v>80</v>
+      </c>
+      <c r="E9" s="4">
+        <f t="shared" si="0"/>
+        <v>180</v>
+      </c>
+      <c r="F9" s="4">
+        <f t="shared" si="3"/>
+        <v>30</v>
+      </c>
+      <c r="G9" s="4">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="24">
+        <v>7</v>
+      </c>
+      <c r="C10" s="42">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="D10" s="4">
+        <v>125</v>
+      </c>
+      <c r="E10" s="4">
+        <f t="shared" si="0"/>
+        <v>225</v>
+      </c>
+      <c r="F10" s="4">
+        <f t="shared" si="3"/>
+        <v>32.1</v>
+      </c>
+      <c r="G10" s="4">
+        <f t="shared" si="2"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="69">
+        <v>8</v>
+      </c>
+      <c r="C11" s="70">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="D11" s="71">
+        <v>200</v>
+      </c>
+      <c r="E11" s="71">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="F11" s="71">
+        <f t="shared" si="3"/>
+        <v>37.5</v>
+      </c>
+      <c r="G11" s="71">
+        <f>E11-E10</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="24">
+        <v>9</v>
+      </c>
+      <c r="C12" s="4">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="D12" s="4">
+        <v>201</v>
+      </c>
+      <c r="E12" s="4">
+        <f t="shared" ref="E12:E13" si="4">C12+D12</f>
+        <v>301</v>
+      </c>
+      <c r="F12" s="4">
+        <f t="shared" ref="F12:F13" si="5">ROUNDDOWN(E12/B12,1)</f>
+        <v>33.4</v>
+      </c>
+      <c r="G12" s="4">
+        <f t="shared" ref="G12:G13" si="6">E12-E11</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="72">
+        <v>10</v>
+      </c>
+      <c r="C13" s="73">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="D13" s="73">
+        <v>202</v>
+      </c>
+      <c r="E13" s="73">
+        <f t="shared" si="4"/>
+        <v>302</v>
+      </c>
+      <c r="F13" s="73">
+        <f t="shared" si="5"/>
+        <v>30.2</v>
+      </c>
+      <c r="G13" s="73">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C16">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B351482E-B0ED-4D3C-A8D2-34B53834CE6E}">
   <dimension ref="B1:F12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3471,11 +3812,11 @@
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
-      <c r="E11" s="69">
+      <c r="E11" s="49">
         <f>Costi!G11</f>
         <v>75</v>
       </c>
-      <c r="F11" s="51" t="str">
+      <c r="F11" s="48" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -3486,7 +3827,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55F4C1D9-4468-40EE-AEC1-05AC83165741}">
   <dimension ref="B1:H13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3743,7 +4084,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A626EAAB-1106-4797-A563-A5DAD61BAF0D}">
   <dimension ref="C2:K22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>